<commit_message>
Fix deliverable bugs: PDF env catalogue, business case schema, BOM SKUs, drawio
- oci_pdf_gen.py: auto-detect new env catalogue schema (name/sizing/cost_pct)
- business-case-spec.yaml: rewritten to match oci_bizcase_gen.py expected
  schema (tco.current_state/proposed_oci with annual_* fields, roi with
  three_year_roi_pct/total_investment/annual_net_benefit, value_drivers
  with category/driver/quantification, roadmap.phases, recommendation.summary)
- bom-spec.yaml: all SKUs verified against oci-sku-catalog.yaml (B110627
  B110629 B110632 for ExaCS X11M, B95703 for ADB-S BYOL, B88326 for
  FastConnect 10G, B91628 for Object Storage, B92092 for Vault)
- diagram-spec.yaml: full dual-region architecture (231 cells, 15 services)
- Now generates: PharmaCorp business case 11 slides, correct env catalogue
  in PDF, 13 SKU lines in BOM with real prices

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/output-demo-pharma-mx/opt14-bom-appca.xlsx
+++ b/examples/output-demo-pharma-mx/opt14-bom-appca.xlsx
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -549,11 +549,11 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>B92459</t>
+          <t>B110627</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>744</v>
@@ -578,11 +578,11 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>B92460</t>
+          <t>B110629</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>744</v>
@@ -607,11 +607,11 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>B97472</t>
+          <t>B110632</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>32</v>
+        <v>128</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>744</v>
@@ -636,14 +636,14 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>B91628</t>
+          <t>B110627</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>50000</v>
+        <v>2</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>1</v>
+        <v>744</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>12</v>
@@ -665,11 +665,11 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>B91960</t>
+          <t>B110629</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>744</v>
@@ -694,27 +694,230 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>B92098</t>
+          <t>B110632</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
+        <v>128</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>744</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>B95703</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>744</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>B95706</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>B88326</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>744</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>B88326</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>744</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>B91628</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>50000</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>B91961</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>B92092</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C15" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="D15" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -734,7 +937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C1:L7"/>
+  <dimension ref="C1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="3" max="3"/>
@@ -884,6 +1087,550 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>B91961</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>OCI - Block Volume Storage</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Gigabyte Storage Capacity Per Month</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>0.0255</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="10">
+        <f>(F8*G8*H8)</f>
+        <v/>
+      </c>
+      <c r="L8" s="10">
+        <f>IFERROR(K8*(1-J8),K8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Oracle Cloud Infrastructure - Autonomous Database &amp; Exadata</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="7" t="n"/>
+      <c r="J9" s="7" t="n"/>
+      <c r="K9" s="7" t="n"/>
+      <c r="L9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>B95703</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Oracle Autonomous Database (ATP or ADW) - BYOL ECPU (2 ECPU minimum)</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>ECPU Per Hour</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>0.08069999999999999</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>744</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="10">
+        <f>(F10*G10*H10)</f>
+        <v/>
+      </c>
+      <c r="L10" s="10">
+        <f>IFERROR(K10*(1-J10),K10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>B95706</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Oracle Autonomous Database Storage for Transaction Processing (ATP), using ECPU</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Gigabyte Storage Capacity Per Month</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>0.1156</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="10">
+        <f>(F11*G11*H11)</f>
+        <v/>
+      </c>
+      <c r="L11" s="10">
+        <f>IFERROR(K11*(1-J11),K11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Oracle Cloud Infrastructure - Database Exadata Infrastructure</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="7" t="n"/>
+      <c r="I12" s="7" t="n"/>
+      <c r="J12" s="7" t="n"/>
+      <c r="K12" s="7" t="n"/>
+      <c r="L12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>B110627</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>OCI - Exadata Cloud Infrastructure - Database Server - X11M</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Hosted Environment Per Hour</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>2.9032</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>744</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="10">
+        <f>(F13*G13*H13)</f>
+        <v/>
+      </c>
+      <c r="L13" s="10">
+        <f>IFERROR(K13*(1-J13),K13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>B110629</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>OCI - Exadata Cloud Infrastructure - Storage Server - X11M</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Hosted Environment Per Hour</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>2.9032</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>744</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="10">
+        <f>(F14*G14*H14)</f>
+        <v/>
+      </c>
+      <c r="L14" s="10">
+        <f>IFERROR(K14*(1-J14),K14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>B110632</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>OCI - Exadata Database ECPU - Dedicated Infrastructure - BYOL (X11M)</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>ECPU Per Hour</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>0.08069999999999999</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>744</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>128</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="J15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="10">
+        <f>(F15*G15*H15)</f>
+        <v/>
+      </c>
+      <c r="L15" s="10">
+        <f>IFERROR(K15*(1-J15),K15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>B110627</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>OCI - Exadata Cloud Infrastructure - Database Server - X11M</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Hosted Environment Per Hour</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>2.9032</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>744</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="10">
+        <f>(F16*G16*H16)</f>
+        <v/>
+      </c>
+      <c r="L16" s="10">
+        <f>IFERROR(K16*(1-J16),K16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>B110629</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>OCI - Exadata Cloud Infrastructure - Storage Server - X11M</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Hosted Environment Per Hour</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>2.9032</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>744</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="J17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="10">
+        <f>(F17*G17*H17)</f>
+        <v/>
+      </c>
+      <c r="L17" s="10">
+        <f>IFERROR(K17*(1-J17),K17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>B110632</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>OCI - Exadata Database ECPU - Dedicated Infrastructure - BYOL (X11M)</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>ECPU Per Hour</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>0.08069999999999999</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>744</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>128</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="J18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="10">
+        <f>(F18*G18*H18)</f>
+        <v/>
+      </c>
+      <c r="L18" s="10">
+        <f>IFERROR(K18*(1-J18),K18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Oracle Cloud Infrastructure - Networking</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="7" t="n"/>
+      <c r="G19" s="7" t="n"/>
+      <c r="H19" s="7" t="n"/>
+      <c r="I19" s="7" t="n"/>
+      <c r="J19" s="7" t="n"/>
+      <c r="K19" s="7" t="n"/>
+      <c r="L19" s="7" t="n"/>
+    </row>
+    <row r="20">
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>B88326</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>OCI - FastConnect 10 Gbps</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Port Hour</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>1.275</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>744</v>
+      </c>
+      <c r="H20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="10">
+        <f>(F20*G20*H20)</f>
+        <v/>
+      </c>
+      <c r="L20" s="10">
+        <f>IFERROR(K20*(1-J20),K20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>B88326</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>OCI - FastConnect 10 Gbps</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Port Hour</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="n">
+        <v>1.275</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>744</v>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="J21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="10">
+        <f>(F21*G21*H21)</f>
+        <v/>
+      </c>
+      <c r="L21" s="10">
+        <f>IFERROR(K21*(1-J21),K21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="C22" s="7" t="n"/>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Oracle Cloud Infrastructure - Security</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="n"/>
+      <c r="F22" s="7" t="n"/>
+      <c r="G22" s="7" t="n"/>
+      <c r="H22" s="7" t="n"/>
+      <c r="I22" s="7" t="n"/>
+      <c r="J22" s="7" t="n"/>
+      <c r="K22" s="7" t="n"/>
+      <c r="L22" s="7" t="n"/>
+    </row>
+    <row r="23">
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>B92092</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>OCI - KMS Vault - Key Versions (Free Tier: 20 Key Versions)</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Key Version Per Month</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>0.5334</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="I23" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="10">
+        <f>(F23*G23*H23)</f>
+        <v/>
+      </c>
+      <c r="L23" s="10">
+        <f>IFERROR(K23*(1-J23),K23)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix BOM: apply global discount_pct from metadata to all line items
oci_bom_gen.py from_spec now reads metadata.discount_pct as fallback
when individual line items don't specify a discount. This means
discount_pct: 0.45 in the spec metadata applies 45% to every SKU.

Previously, global discount was silently ignored — only per-item
discount fields were read (defaulting to 0.0).

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/output-demo-pharma-mx/opt14-bom-appca.xlsx
+++ b/examples/output-demo-pharma-mx/opt14-bom-appca.xlsx
@@ -562,7 +562,7 @@
         <v>12</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
@@ -591,7 +591,7 @@
         <v>12</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
@@ -620,7 +620,7 @@
         <v>12</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
@@ -649,7 +649,7 @@
         <v>12</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
@@ -678,7 +678,7 @@
         <v>12</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
@@ -707,7 +707,7 @@
         <v>12</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
@@ -736,7 +736,7 @@
         <v>12</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
@@ -765,7 +765,7 @@
         <v>12</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
@@ -794,7 +794,7 @@
         <v>12</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
         <v>12</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
@@ -852,7 +852,7 @@
         <v>12</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
@@ -881,7 +881,7 @@
         <v>12</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
@@ -910,7 +910,7 @@
         <v>12</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
@@ -1076,7 +1076,7 @@
         <v>12</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="K7" s="10">
         <f>(F7*G7*H7)</f>
@@ -1116,7 +1116,7 @@
         <v>12</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="K8" s="10">
         <f>(F8*G8*H8)</f>
@@ -1172,7 +1172,7 @@
         <v>12</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="K10" s="10">
         <f>(F10*G10*H10)</f>
@@ -1212,7 +1212,7 @@
         <v>12</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="K11" s="10">
         <f>(F11*G11*H11)</f>
@@ -1268,7 +1268,7 @@
         <v>12</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="K13" s="10">
         <f>(F13*G13*H13)</f>
@@ -1308,7 +1308,7 @@
         <v>12</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="K14" s="10">
         <f>(F14*G14*H14)</f>
@@ -1348,7 +1348,7 @@
         <v>12</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="K15" s="10">
         <f>(F15*G15*H15)</f>
@@ -1388,7 +1388,7 @@
         <v>12</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="K16" s="10">
         <f>(F16*G16*H16)</f>
@@ -1428,7 +1428,7 @@
         <v>12</v>
       </c>
       <c r="J17" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="K17" s="10">
         <f>(F17*G17*H17)</f>
@@ -1468,7 +1468,7 @@
         <v>12</v>
       </c>
       <c r="J18" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="K18" s="10">
         <f>(F18*G18*H18)</f>
@@ -1524,7 +1524,7 @@
         <v>12</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="K20" s="10">
         <f>(F20*G20*H20)</f>
@@ -1564,7 +1564,7 @@
         <v>12</v>
       </c>
       <c r="J21" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="K21" s="10">
         <f>(F21*G21*H21)</f>
@@ -1620,7 +1620,7 @@
         <v>12</v>
       </c>
       <c r="J23" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="K23" s="10">
         <f>(F23*G23*H23)</f>

</xml_diff>